<commit_message>
Actualización de archivos JSON y scripts 09 de marzo 2026
</commit_message>
<xml_diff>
--- a/Colmedica.xlsx
+++ b/Colmedica.xlsx
@@ -438,7 +438,9 @@
 19/09/2025 Lectura del encabezado para ir sacando el registro tipo 1 (Encabezado)
 25/02/2026 se retoma, el desarrollo dandole un vuelco para unificar el código y dejarlo de manera virtual
 26/02/2026 ajustes a la pagina a conexiones de bases de datos dependiendo de la base donde se encuentre la tabla
-27/02/2026 Ajuste de ciclos y querys según las funciones y/o clases defindas en la conexión ya existente. Ya no genera error el código, pero se le está haciendo seguimiento a los querys y ejecución para obtener el resultado de los respectivos archivos</t>
+27/02/2026 Ajuste de ciclos y querys según las funciones y/o clases defindas en la conexión ya existente. Ya no genera error el código, pero se le está haciendo seguimiento a los querys y ejecución para obtener el resultado de los respectivos archivos
+6/03/2026 se terminaron de ajustar los errores de la pagina en la generación de afiliaciones nuevas
+9/03/2026 se empiezan a validar inconsistencias para la generación de Inclusiones. y como ya se generan archivos, pues se debe realizar la comparación de estructura y data con la generada actualmente por el access</t>
   </si>
   <si>
     <t>OPT_7</t>
@@ -3947,7 +3949,7 @@
         <v>95</v>
       </c>
       <c r="G22" s="23">
-        <v>50</v>
+        <v>85</v>
       </c>
       <c r="H22" s="24">
         <f>IF(OR(J22="",K22="",K22&lt;J22),0,NETWORKDAYS(J22,K22,Hoja2!$A$2:$A$53))</f>
@@ -3970,7 +3972,7 @@
       NETWORKDAYS(J22,L22,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N22" s="28"/>
       <c r="O22" s="28"/>
@@ -4124,7 +4126,7 @@
       NETWORKDAYS(J24,L24,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N24" s="28"/>
       <c r="O24" s="28"/>
@@ -4914,7 +4916,7 @@
       NETWORKDAYS(J34,L34,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="N34" s="28"/>
       <c r="O34" s="28"/>
@@ -5230,7 +5232,7 @@
       NETWORKDAYS(J38,L38,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="N38" s="28"/>
       <c r="O38" s="28"/>

</xml_diff>

<commit_message>
Actualización de archivos JSON y scripts 12 de marzo 2026
</commit_message>
<xml_diff>
--- a/Colmedica.xlsx
+++ b/Colmedica.xlsx
@@ -858,7 +858,8 @@
 11/02/2026 Se validan los filtros solicitados sobre los campos para consultas puntuales
 27/02/2026 se confirman, cambios, y se informa al cliente para la revisión
 3/03/2026 se hace reunión con el átrea para hacer retroalimentación, y piden unos ajustes de forma para poder pasar a producción
-4/03/2026 se empiezan a hacer los ajustes solicitados en la reunión anterioir</t>
+4/03/2026 se empiezan a hacer los ajustes solicitados en la reunión anterioir
+10/03/2026 se hace reunión para mostrar los ajustes según la última reunión, y se aprueban por parte del área para paso a producción</t>
   </si>
   <si>
     <t>OPT_22</t>
@@ -3972,7 +3973,7 @@
       NETWORKDAYS(J22,L22,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N22" s="28"/>
       <c r="O22" s="28"/>
@@ -4126,7 +4127,7 @@
       NETWORKDAYS(J24,L24,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="N24" s="28"/>
       <c r="O24" s="28"/>
@@ -4916,7 +4917,7 @@
       NETWORKDAYS(J34,L34,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="N34" s="28"/>
       <c r="O34" s="28"/>
@@ -5232,7 +5233,7 @@
       NETWORKDAYS(J38,L38,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="N38" s="28"/>
       <c r="O38" s="28"/>
@@ -6269,10 +6270,10 @@
       </c>
       <c r="E52" s="21"/>
       <c r="F52" s="22" t="s">
-        <v>95</v>
+        <v>21</v>
       </c>
       <c r="G52" s="23">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H52" s="24">
         <f>IF(OR(J52="",K52="",K52&lt;J52),0,NETWORKDAYS(J52,K52,Hoja2!$A$2:$A$53))</f>
@@ -6303,7 +6304,9 @@
       <c r="O52" s="28">
         <v>46080</v>
       </c>
-      <c r="P52" s="28"/>
+      <c r="P52" s="28">
+        <v>46091</v>
+      </c>
       <c r="Q52" s="29" t="s">
         <v>212</v>
       </c>

</xml_diff>

<commit_message>
Actualización de archivos JSON y scripts 24 de junio 2026
</commit_message>
<xml_diff>
--- a/Colmedica.xlsx
+++ b/Colmedica.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7455"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12135"/>
   </bookViews>
   <sheets>
     <sheet name="EN PROCESO (Colmedica)" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="pruebas i" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EN PROCESO (Colmedica)'!$A$1:$R$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EN PROCESO (Colmedica)'!$A$1:$R$80</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1390" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1397" uniqueCount="383">
   <si>
     <t>Asignado a</t>
   </si>
@@ -1102,7 +1102,8 @@
     <t>25/05/2026 Se entrega documento con el requerimiento a Don HErnán y el crea la opción
 26/05/2026 Se piden ajustes sobre la información pintada en pantalla y y se realizan primeras pruebas de subir soportes
 27/05/2026 se solicita una adición de validación a la cantidad de folios, y se pide nuevamente ajustes a la  pantalla principal que muestra información innecesaria y satura la vista
-28/05/2026 Se confirma que puede ser entregado el proyecto para ponerlo en desarrollo y empezar a hacer los ajsutes relacionados a conexión base de datos y url destino de las imágenes adecuadas al servidor</t>
+28/05/2026 Se confirma que puede ser entregado el proyecto para ponerlo en desarrollo y empezar a hacer los ajsutes relacionados a conexión base de datos
+23/06/2026 Se explica a Jhon, para ajuste de url destino de las imágenes adecuadas al servidor, y que no cargeu pagina de logueo, sino que se incoque el usuario del logueo incial y se lleve a ese link</t>
   </si>
   <si>
     <t>OPT_50</t>
@@ -1132,31 +1133,44 @@
     <t>Informe soporte para la Facturacion, Registros de Gestión durante el mes y registros de causales de acreditación durante el mes</t>
   </si>
   <si>
+    <t>OPT_53</t>
+  </si>
+  <si>
+    <t>Tutelas - Ajuste de Visor Imagenes</t>
+  </si>
+  <si>
+    <t>Ajustar el visor para ver imágenes tiff,pdf,jpg,png</t>
+  </si>
+  <si>
+    <t>18/06/2026 se evalua y revisa el visor actual de las archivos que se suben de tutelas y se inicia el ajuste según visro actual de afiliaciones
+19/06/2026 se pasa a pruebas y se informa al cliente para que revisen la visualización</t>
+  </si>
+  <si>
     <t>Afiliaciones POS - Completar descarga de cartas Derechos y Deberes</t>
   </si>
   <si>
+    <t>19/11/2025 Posible mejora detectada por Imagine -Jennifer</t>
+  </si>
+  <si>
     <t>Afiliaciones Pre - Llegan casos con imágenes repetidas en el xml, generando imágenes incompletas en el proceso</t>
   </si>
   <si>
     <t>Opción para eliminar imágenes duplicadas dentro de la ya actual de reproceso de Afiliaciones Pre</t>
   </si>
   <si>
-    <t>19/11/2025 Posible mejora detectada por Imagine -Jennifer</t>
-  </si>
-  <si>
     <t>Afiliaciones POS - Consumo Puntual de las afiliaciones</t>
   </si>
   <si>
     <t>Acreditación - Validación de casos para saber su ultima acreditacion Desarrollo</t>
   </si>
   <si>
+    <t>01/2026 Posible mejora detectada por Imagine -Jennifer</t>
+  </si>
+  <si>
     <t>Convenios Medicos - Cargue Masivo de Planes a Nits</t>
   </si>
   <si>
     <t>Cargue de excel para relacionar de manera masiva los planes creados nuevos por Colmédica a los diferentes prestadores</t>
-  </si>
-  <si>
-    <t>01/2026 Posible mejora detectada por Imagine -Jennifer</t>
   </si>
   <si>
     <t>Afiliaciones POS - Cargue de SAT</t>
@@ -2460,7 +2474,7 @@
   <sheetPr>
     <tabColor rgb="FF93C47D"/>
   </sheetPr>
-  <dimension ref="A1:AN79"/>
+  <dimension ref="A1:AN80"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.21875" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="8.109375" customWidth="1"/>
@@ -4134,7 +4148,7 @@
       NETWORKDAYS(J21,L21,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="N21" s="43"/>
       <c r="O21" s="43">
@@ -4292,7 +4306,7 @@
       NETWORKDAYS(J23,L23,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="N23" s="43"/>
       <c r="O23" s="43"/>
@@ -5084,7 +5098,7 @@
       NETWORKDAYS(J33,L33,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="N33" s="43"/>
       <c r="O33" s="43"/>
@@ -5473,7 +5487,7 @@
       NETWORKDAYS(J38,L38,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="N38" s="28"/>
       <c r="O38" s="28">
@@ -6929,7 +6943,7 @@
       NETWORKDAYS(J56,L56,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="N56" s="28"/>
       <c r="O56" s="28">
@@ -7008,7 +7022,7 @@
       NETWORKDAYS(J57,L57,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="N57" s="43"/>
       <c r="O57" s="43">
@@ -7087,7 +7101,7 @@
       NETWORKDAYS(J58,L58,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="N58" s="28"/>
       <c r="O58" s="28">
@@ -7164,7 +7178,7 @@
       NETWORKDAYS(J59,L59,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="N59" s="43"/>
       <c r="O59" s="43"/>
@@ -7644,7 +7658,7 @@
       NETWORKDAYS(J65,L65,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="N65" s="43"/>
       <c r="O65" s="43">
@@ -7723,7 +7737,7 @@
       NETWORKDAYS(J66,L66,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="N66" s="28"/>
       <c r="O66" s="28">
@@ -7869,7 +7883,7 @@
       NETWORKDAYS(J68,L68,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="N68" s="28"/>
       <c r="O68" s="28"/>
@@ -7942,7 +7956,7 @@
       NETWORKDAYS(J69,L69,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="N69" s="43"/>
       <c r="O69" s="43"/>
@@ -8114,29 +8128,39 @@
       <c r="AM71" s="60"/>
       <c r="AN71" s="61"/>
     </row>
-    <row r="72" spans="1:40" ht="57">
+    <row r="72" spans="1:40" ht="28.5">
       <c r="A72" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="B72" s="18"/>
+      <c r="B72" s="18" t="s">
+        <v>288</v>
+      </c>
       <c r="C72" s="19" t="s">
-        <v>288</v>
-      </c>
-      <c r="D72" s="20"/>
+        <v>289</v>
+      </c>
+      <c r="D72" s="20" t="s">
+        <v>290</v>
+      </c>
       <c r="E72" s="21"/>
       <c r="F72" s="22" t="s">
-        <v>110</v>
+        <v>91</v>
       </c>
       <c r="G72" s="23">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H72" s="24">
         <f>IF(OR(J72="",K72="",K72&lt;J72),0,NETWORKDAYS(J72,K72,Hoja2!$A$2:$A$53))</f>
-        <v>0</v>
-      </c>
-      <c r="I72" s="25"/>
-      <c r="J72" s="25"/>
-      <c r="K72" s="26"/>
+        <v>2</v>
+      </c>
+      <c r="I72" s="25">
+        <v>46190</v>
+      </c>
+      <c r="J72" s="25">
+        <v>46191</v>
+      </c>
+      <c r="K72" s="26">
+        <v>46192</v>
+      </c>
       <c r="L72" s="26"/>
       <c r="M72" s="27">
         <f ca="1">IF(OR(J72="",AND(L72="",TODAY()&lt;J72),AND(L72&lt;&gt;"",L72&lt;J72)),0,
@@ -8145,12 +8169,16 @@
       NETWORKDAYS(J72,L72,Hoja2!$A$2:$A$53)
    )
 )</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N72" s="28"/>
-      <c r="O72" s="28"/>
+      <c r="O72" s="28">
+        <v>46192</v>
+      </c>
       <c r="P72" s="28"/>
-      <c r="Q72" s="29"/>
+      <c r="Q72" s="29" t="s">
+        <v>291</v>
+      </c>
       <c r="R72" s="30" t="s">
         <v>102</v>
       </c>
@@ -8177,17 +8205,15 @@
       <c r="AM72" s="62"/>
       <c r="AN72" s="63"/>
     </row>
-    <row r="73" spans="1:40" ht="71.25">
+    <row r="73" spans="1:40" ht="57">
       <c r="A73" s="32" t="s">
         <v>37</v>
       </c>
       <c r="B73" s="33"/>
       <c r="C73" s="34" t="s">
-        <v>289</v>
-      </c>
-      <c r="D73" s="35" t="s">
-        <v>290</v>
-      </c>
+        <v>292</v>
+      </c>
+      <c r="D73" s="35"/>
       <c r="E73" s="36"/>
       <c r="F73" s="37" t="s">
         <v>110</v>
@@ -8216,7 +8242,7 @@
       <c r="O73" s="43"/>
       <c r="P73" s="43"/>
       <c r="Q73" s="44" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="R73" s="45" t="s">
         <v>102</v>
@@ -8244,15 +8270,17 @@
       <c r="AM73" s="60"/>
       <c r="AN73" s="61"/>
     </row>
-    <row r="74" spans="1:40" ht="42.75">
+    <row r="74" spans="1:40" ht="71.25">
       <c r="A74" s="17" t="s">
         <v>37</v>
       </c>
       <c r="B74" s="18"/>
       <c r="C74" s="19" t="s">
-        <v>292</v>
-      </c>
-      <c r="D74" s="20"/>
+        <v>294</v>
+      </c>
+      <c r="D74" s="20" t="s">
+        <v>295</v>
+      </c>
       <c r="E74" s="21"/>
       <c r="F74" s="22" t="s">
         <v>110</v>
@@ -8307,11 +8335,11 @@
       <c r="AM74" s="62"/>
       <c r="AN74" s="63"/>
     </row>
-    <row r="75" spans="1:40" ht="57">
+    <row r="75" spans="1:40" ht="42.75">
       <c r="A75" s="32"/>
       <c r="B75" s="33"/>
       <c r="C75" s="34" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="D75" s="35"/>
       <c r="E75" s="36"/>
@@ -8368,15 +8396,13 @@
       <c r="AM75" s="60"/>
       <c r="AN75" s="61"/>
     </row>
-    <row r="76" spans="1:40" ht="71.25">
+    <row r="76" spans="1:40" ht="57">
       <c r="A76" s="17"/>
       <c r="B76" s="18"/>
       <c r="C76" s="19" t="s">
-        <v>289</v>
-      </c>
-      <c r="D76" s="20" t="s">
-        <v>290</v>
-      </c>
+        <v>297</v>
+      </c>
+      <c r="D76" s="20"/>
       <c r="E76" s="21"/>
       <c r="F76" s="22" t="s">
         <v>110</v>
@@ -8405,7 +8431,7 @@
       <c r="O76" s="28"/>
       <c r="P76" s="28"/>
       <c r="Q76" s="29" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="R76" s="30" t="s">
         <v>102</v>
@@ -8433,13 +8459,15 @@
       <c r="AM76" s="62"/>
       <c r="AN76" s="63"/>
     </row>
-    <row r="77" spans="1:40" ht="42.75">
+    <row r="77" spans="1:40" ht="71.25">
       <c r="A77" s="32"/>
       <c r="B77" s="33"/>
       <c r="C77" s="34" t="s">
-        <v>292</v>
-      </c>
-      <c r="D77" s="35"/>
+        <v>294</v>
+      </c>
+      <c r="D77" s="35" t="s">
+        <v>295</v>
+      </c>
       <c r="E77" s="36"/>
       <c r="F77" s="37" t="s">
         <v>110</v>
@@ -8498,11 +8526,9 @@
       <c r="A78" s="17"/>
       <c r="B78" s="18"/>
       <c r="C78" s="19" t="s">
-        <v>294</v>
-      </c>
-      <c r="D78" s="20" t="s">
-        <v>295</v>
-      </c>
+        <v>296</v>
+      </c>
+      <c r="D78" s="20"/>
       <c r="E78" s="21"/>
       <c r="F78" s="22" t="s">
         <v>110</v>
@@ -8531,7 +8557,7 @@
       <c r="O78" s="28"/>
       <c r="P78" s="28"/>
       <c r="Q78" s="29" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="R78" s="30" t="s">
         <v>102</v>
@@ -8559,16 +8585,16 @@
       <c r="AM78" s="62"/>
       <c r="AN78" s="63"/>
     </row>
-    <row r="79" spans="1:40" ht="38.25">
+    <row r="79" spans="1:40" ht="42.75">
       <c r="A79" s="32" t="s">
         <v>37</v>
       </c>
       <c r="B79" s="33"/>
       <c r="C79" s="34" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D79" s="35" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="E79" s="36"/>
       <c r="F79" s="37" t="s">
@@ -8598,7 +8624,7 @@
       <c r="O79" s="43"/>
       <c r="P79" s="43"/>
       <c r="Q79" s="44" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="R79" s="45" t="s">
         <v>102</v>
@@ -8626,18 +8652,83 @@
       <c r="AM79" s="60"/>
       <c r="AN79" s="61"/>
     </row>
+    <row r="80" spans="1:40" ht="38.25">
+      <c r="A80" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B80" s="18"/>
+      <c r="C80" s="19" t="s">
+        <v>301</v>
+      </c>
+      <c r="D80" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="E80" s="21"/>
+      <c r="F80" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="G80" s="23">
+        <v>0</v>
+      </c>
+      <c r="H80" s="24">
+        <f>IF(OR(J80="",K80="",K80&lt;J80),0,NETWORKDAYS(J80,K80,Hoja2!$A$2:$A$53))</f>
+        <v>0</v>
+      </c>
+      <c r="I80" s="69"/>
+      <c r="J80" s="50"/>
+      <c r="K80" s="28"/>
+      <c r="L80" s="28"/>
+      <c r="M80" s="27">
+        <f ca="1">IF(OR(J80="",AND(L80="",TODAY()&lt;J80),AND(L80&lt;&gt;"",L80&lt;J80)),0,
+   IF(L80="",
+      NETWORKDAYS(J80,TODAY(),Hoja2!$A$2:$A$53),
+      NETWORKDAYS(J80,L80,Hoja2!$A$2:$A$53)
+   )
+)</f>
+        <v>0</v>
+      </c>
+      <c r="N80" s="28"/>
+      <c r="O80" s="28"/>
+      <c r="P80" s="28"/>
+      <c r="Q80" s="29"/>
+      <c r="R80" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="S80" s="62"/>
+      <c r="T80" s="62"/>
+      <c r="U80" s="62"/>
+      <c r="V80" s="62"/>
+      <c r="W80" s="62"/>
+      <c r="X80" s="62"/>
+      <c r="Y80" s="62"/>
+      <c r="Z80" s="62"/>
+      <c r="AA80" s="62"/>
+      <c r="AB80" s="62"/>
+      <c r="AC80" s="62"/>
+      <c r="AD80" s="62"/>
+      <c r="AE80" s="62"/>
+      <c r="AF80" s="62"/>
+      <c r="AG80" s="62"/>
+      <c r="AH80" s="62"/>
+      <c r="AI80" s="62"/>
+      <c r="AJ80" s="62"/>
+      <c r="AK80" s="62"/>
+      <c r="AL80" s="62"/>
+      <c r="AM80" s="62"/>
+      <c r="AN80" s="63"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R79"/>
+  <autoFilter ref="A1:R80"/>
   <conditionalFormatting sqref="B7:B79">
     <cfRule type="expression" dxfId="0" priority="2">
-      <formula>COUNTIF(B7:B79, B7)&gt;1</formula>
+      <formula>COUNTIF(B7:B80, B7)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:L25 N2:P25 I26 I27:L79 N27:P79">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:L25 N2:P25 I26 I27:L80 N27:P80">
       <formula1>OR(NOT(ISERROR(DATEVALUE(I2))), AND(ISNUMBER(I2), LEFT(CELL("format", I2))="D"))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F79">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F80">
       <formula1>"FINALIZADO,EN PROCESO,PAUSADO,EN TEST,PENDIENTE,PRUEBAS CLIENTE,PRUEBAS IMAGINE,PASO A PRODUCCION,PENDIENTE CLIENTE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8659,7 +8750,7 @@
         <v>45292</v>
       </c>
       <c r="B1" s="72" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="17.25" customHeight="1">
@@ -8667,7 +8758,7 @@
         <v>45299</v>
       </c>
       <c r="B2" s="72" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="17.25" customHeight="1">
@@ -8675,7 +8766,7 @@
         <v>45376</v>
       </c>
       <c r="B3" s="72" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="17.25" customHeight="1">
@@ -8683,7 +8774,7 @@
         <v>45379</v>
       </c>
       <c r="B4" s="72" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="17.25" customHeight="1">
@@ -8691,7 +8782,7 @@
         <v>45380</v>
       </c>
       <c r="B5" s="72" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="17.25" customHeight="1">
@@ -8699,7 +8790,7 @@
         <v>45413</v>
       </c>
       <c r="B6" s="72" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="17.25" customHeight="1">
@@ -8707,7 +8798,7 @@
         <v>45425</v>
       </c>
       <c r="B7" s="72" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="17.25" customHeight="1">
@@ -8715,7 +8806,7 @@
         <v>45446</v>
       </c>
       <c r="B8" s="72" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="17.25" customHeight="1">
@@ -8723,7 +8814,7 @@
         <v>45453</v>
       </c>
       <c r="B9" s="72" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="17.25" customHeight="1">
@@ -8731,7 +8822,7 @@
         <v>45474</v>
       </c>
       <c r="B10" s="72" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="17.25" customHeight="1">
@@ -8739,7 +8830,7 @@
         <v>45493</v>
       </c>
       <c r="B11" s="72" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="17.25" customHeight="1">
@@ -8747,7 +8838,7 @@
         <v>45511</v>
       </c>
       <c r="B12" s="72" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="17.25" customHeight="1">
@@ -8755,7 +8846,7 @@
         <v>45523</v>
       </c>
       <c r="B13" s="72" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="17.25" customHeight="1">
@@ -8763,7 +8854,7 @@
         <v>45579</v>
       </c>
       <c r="B14" s="72" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="17.25" customHeight="1">
@@ -8771,7 +8862,7 @@
         <v>45600</v>
       </c>
       <c r="B15" s="72" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="17.25" customHeight="1">
@@ -8779,7 +8870,7 @@
         <v>45607</v>
       </c>
       <c r="B16" s="72" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="17.25" customHeight="1">
@@ -8787,7 +8878,7 @@
         <v>45634</v>
       </c>
       <c r="B17" s="72" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="17.25" customHeight="1">
@@ -8795,7 +8886,7 @@
         <v>45651</v>
       </c>
       <c r="B18" s="72" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="17.25" customHeight="1">
@@ -8803,7 +8894,7 @@
         <v>45658</v>
       </c>
       <c r="B19" s="73" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="17.25" customHeight="1">
@@ -8811,7 +8902,7 @@
         <v>45663</v>
       </c>
       <c r="B20" s="73" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="17.25" customHeight="1">
@@ -8819,7 +8910,7 @@
         <v>45740</v>
       </c>
       <c r="B21" s="73" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="17.25" customHeight="1">
@@ -8827,7 +8918,7 @@
         <v>45764</v>
       </c>
       <c r="B22" s="73" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="17.25" customHeight="1">
@@ -8835,7 +8926,7 @@
         <v>45765</v>
       </c>
       <c r="B23" s="73" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="17.25" customHeight="1">
@@ -8843,7 +8934,7 @@
         <v>45778</v>
       </c>
       <c r="B24" s="73" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="17.25" customHeight="1">
@@ -8851,7 +8942,7 @@
         <v>45810</v>
       </c>
       <c r="B25" s="73" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="17.25" customHeight="1">
@@ -8859,7 +8950,7 @@
         <v>45831</v>
       </c>
       <c r="B26" s="73" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="17.25" customHeight="1">
@@ -8867,7 +8958,7 @@
         <v>45838</v>
       </c>
       <c r="B27" s="73" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="17.25" customHeight="1">
@@ -8875,7 +8966,7 @@
         <v>45858</v>
       </c>
       <c r="B28" s="73" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="17.25" customHeight="1">
@@ -8883,7 +8974,7 @@
         <v>45876</v>
       </c>
       <c r="B29" s="73" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="17.25" customHeight="1">
@@ -8891,7 +8982,7 @@
         <v>45887</v>
       </c>
       <c r="B30" s="73" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="17.25" customHeight="1">
@@ -8899,7 +8990,7 @@
         <v>45943</v>
       </c>
       <c r="B31" s="73" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="17.25" customHeight="1">
@@ -8907,7 +8998,7 @@
         <v>45964</v>
       </c>
       <c r="B32" s="73" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="17.25" customHeight="1">
@@ -8915,7 +9006,7 @@
         <v>45978</v>
       </c>
       <c r="B33" s="73" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="17.25" customHeight="1">
@@ -8923,7 +9014,7 @@
         <v>45999</v>
       </c>
       <c r="B34" s="73" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="17.25" customHeight="1">
@@ -8931,7 +9022,7 @@
         <v>46016</v>
       </c>
       <c r="B35" s="73" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="17.25" customHeight="1">
@@ -8939,7 +9030,7 @@
         <v>46023</v>
       </c>
       <c r="B36" s="73" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="17.25" customHeight="1">
@@ -8947,7 +9038,7 @@
         <v>46034</v>
       </c>
       <c r="B37" s="73" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="17.25" customHeight="1">
@@ -8955,7 +9046,7 @@
         <v>46104</v>
       </c>
       <c r="B38" s="73" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="17.25" customHeight="1">
@@ -8963,7 +9054,7 @@
         <v>46114</v>
       </c>
       <c r="B39" s="73" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="17.25" customHeight="1">
@@ -8971,7 +9062,7 @@
         <v>46115</v>
       </c>
       <c r="B40" s="73" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="17.25" customHeight="1">
@@ -8979,7 +9070,7 @@
         <v>46143</v>
       </c>
       <c r="B41" s="73" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="17.25" customHeight="1">
@@ -8987,7 +9078,7 @@
         <v>46160</v>
       </c>
       <c r="B42" s="73" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="17.25" customHeight="1">
@@ -8995,7 +9086,7 @@
         <v>46181</v>
       </c>
       <c r="B43" s="73" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="17.25" customHeight="1">
@@ -9003,7 +9094,7 @@
         <v>46188</v>
       </c>
       <c r="B44" s="73" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="17.25" customHeight="1">
@@ -9011,7 +9102,7 @@
         <v>46202</v>
       </c>
       <c r="B45" s="73" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="17.25" customHeight="1">
@@ -9019,7 +9110,7 @@
         <v>46223</v>
       </c>
       <c r="B46" s="73" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="17.25" customHeight="1">
@@ -9027,7 +9118,7 @@
         <v>46241</v>
       </c>
       <c r="B47" s="73" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="17.25" customHeight="1">
@@ -9035,7 +9126,7 @@
         <v>46251</v>
       </c>
       <c r="B48" s="73" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="17.25" customHeight="1">
@@ -9043,7 +9134,7 @@
         <v>46307</v>
       </c>
       <c r="B49" s="73" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="17.25" customHeight="1">
@@ -9051,7 +9142,7 @@
         <v>46328</v>
       </c>
       <c r="B50" s="73" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="17.25" customHeight="1">
@@ -9059,7 +9150,7 @@
         <v>46342</v>
       </c>
       <c r="B51" s="73" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="17.25" customHeight="1">
@@ -9067,7 +9158,7 @@
         <v>46364</v>
       </c>
       <c r="B52" s="73" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="17.25" customHeight="1">
@@ -9075,7 +9166,7 @@
         <v>46381</v>
       </c>
       <c r="B53" s="73" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="17.25" customHeight="1"/>
@@ -10044,7 +10135,7 @@
   <sheetData>
     <row r="1" spans="1:97" ht="15.75">
       <c r="A1" s="74" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="B1" s="75"/>
       <c r="C1" s="75"/>
@@ -10102,7 +10193,7 @@
     </row>
     <row r="3" spans="1:97" ht="32.25" customHeight="1">
       <c r="A3" s="76" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="B3" s="77">
         <v>45596</v>
@@ -10395,261 +10486,261 @@
     </row>
     <row r="4" spans="1:97" ht="30.75" customHeight="1">
       <c r="A4" s="80" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="B4" s="81" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="C4" s="82" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="D4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="E4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="F4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="G4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="H4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="I4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="J4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="K4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="L4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="M4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="N4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="O4" s="83" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="P4" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Q4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="R4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="S4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="T4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="U4" s="84" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="V4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="W4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="X4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Y4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Z4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AA4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AB4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AC4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AD4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AE4" s="109" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="AF4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AG4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AH4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AI4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AJ4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AK4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AL4" s="109" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="AM4" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AN4" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AO4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AP4" s="109" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="AQ4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AR4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AS4" s="109" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="AT4" s="85" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AU4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AV4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AW4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AX4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AY4" s="109" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="AZ4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BA4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BB4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BC4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BD4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BE4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BF4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BG4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BH4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BI4" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BJ4" s="109" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="BK4" s="84" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="BL4" s="84" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="BM4" s="84" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="BN4" s="84" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="BO4" s="84" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="BP4" s="84" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="BQ4" s="84" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="BR4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BS4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BT4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BU4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BV4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BW4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BX4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BY4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BZ4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CA4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CB4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CC4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CD4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CE4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CF4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CG4" s="83"/>
       <c r="CH4" s="83"/>
       <c r="CI4" s="109" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="CJ4" s="83"/>
       <c r="CK4" s="83"/>
@@ -10661,249 +10752,249 @@
       <c r="CQ4" s="83"/>
       <c r="CR4" s="83"/>
       <c r="CS4" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
     </row>
     <row r="5" spans="1:97" ht="15.75" customHeight="1">
       <c r="A5" s="80" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="B5" s="81" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="C5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="D5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="E5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="F5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="G5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="H5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="I5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="J5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="K5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="L5" s="83" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="M5" s="83" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="N5" s="83" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="O5" s="83" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="P5" s="84" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="Q5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="R5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="S5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="T5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="U5" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="V5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="W5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="X5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Y5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Z5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AA5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AB5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AC5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AD5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AE5" s="110"/>
       <c r="AF5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AG5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AH5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AI5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AJ5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AK5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AL5" s="110"/>
       <c r="AM5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AN5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AO5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AP5" s="110"/>
       <c r="AQ5" s="83" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="AR5" s="83" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="AS5" s="110"/>
       <c r="AT5" s="83" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="AU5" s="83" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="AV5" s="83" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="AW5" s="83" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="AX5" s="83" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="AY5" s="110"/>
       <c r="AZ5" s="83" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="BA5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BB5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BC5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BD5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BE5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BF5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BG5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BH5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BI5" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BJ5" s="110"/>
       <c r="BK5" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BL5" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BM5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BN5" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BO5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BP5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BQ5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BR5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BS5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BT5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BU5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BV5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BW5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BX5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BY5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BZ5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CA5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CB5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CC5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CD5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CE5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CF5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CG5" s="83"/>
       <c r="CH5" s="83"/>
@@ -10918,249 +11009,249 @@
       <c r="CQ5" s="83"/>
       <c r="CR5" s="83"/>
       <c r="CS5" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
     </row>
     <row r="6" spans="1:97" ht="15.75">
       <c r="A6" s="80" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="B6" s="81" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="C6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="D6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="E6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="F6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="G6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="H6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="I6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="J6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="K6" s="86" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="L6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="M6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="N6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="O6" s="83" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="P6" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Q6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="R6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="S6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="T6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="U6" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="V6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="W6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="X6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Y6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Z6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AA6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AB6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AC6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AD6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AE6" s="110"/>
       <c r="AF6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AG6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AH6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AI6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AJ6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AK6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AL6" s="110"/>
       <c r="AM6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AN6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AO6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AP6" s="110"/>
       <c r="AQ6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AR6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AS6" s="110"/>
       <c r="AT6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AU6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AV6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AW6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AX6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AY6" s="110"/>
       <c r="AZ6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BA6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BB6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BC6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BD6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BE6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BF6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BG6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BH6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BI6" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BJ6" s="110"/>
       <c r="BK6" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BL6" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BM6" s="83" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="BN6" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BO6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BP6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BQ6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BR6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BS6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BT6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BU6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BV6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BW6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BX6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BY6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BZ6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CA6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CB6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CC6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CD6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CE6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CF6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CG6" s="83"/>
       <c r="CH6" s="83"/>
@@ -11175,198 +11266,198 @@
       <c r="CQ6" s="83"/>
       <c r="CR6" s="83"/>
       <c r="CS6" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
     </row>
     <row r="7" spans="1:97" ht="15.75" hidden="1" customHeight="1">
       <c r="A7" s="80" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="B7" s="81" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="C7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="D7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="E7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="F7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="G7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="H7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="I7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="J7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="K7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="L7" s="86" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="M7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="N7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="O7" s="83" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="P7" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Q7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="R7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="S7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="T7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="U7" s="84" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="V7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="W7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="X7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Y7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Z7" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AA7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AB7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AC7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AD7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AE7" s="110"/>
       <c r="AF7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AG7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AH7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AI7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AJ7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AK7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AL7" s="110"/>
       <c r="AM7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AN7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AO7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AP7" s="110"/>
       <c r="AQ7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AR7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AS7" s="110"/>
       <c r="AT7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AU7" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AV7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AW7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AX7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AY7" s="110"/>
       <c r="AZ7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BA7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BB7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BC7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BD7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BE7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BF7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BG7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BH7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BI7" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BJ7" s="110"/>
       <c r="BK7" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BL7" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BM7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BN7" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BO7" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BP7" s="83"/>
       <c r="BQ7" s="83"/>
@@ -11374,16 +11465,16 @@
       <c r="BS7" s="83"/>
       <c r="BT7" s="83"/>
       <c r="BU7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BV7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BW7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BX7" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BY7" s="83"/>
       <c r="BZ7" s="83"/>
@@ -11409,220 +11500,220 @@
     </row>
     <row r="8" spans="1:97" ht="15.75" hidden="1" customHeight="1">
       <c r="A8" s="80" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="B8" s="81" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="C8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="D8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="E8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="F8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="G8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="H8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="I8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="J8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="K8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="L8" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="M8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="N8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="O8" s="83" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="P8" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Q8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="R8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="S8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="T8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="U8" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="V8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="W8" s="83" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="X8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Y8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Z8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AA8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AB8" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AC8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AD8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AE8" s="110"/>
       <c r="AF8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AG8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AH8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AI8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AJ8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AK8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AL8" s="110"/>
       <c r="AM8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AN8" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AO8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AP8" s="110"/>
       <c r="AQ8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AR8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AS8" s="110"/>
       <c r="AT8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AU8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AV8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AW8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AX8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AY8" s="110"/>
       <c r="AZ8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BA8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BB8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BC8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BD8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BE8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BF8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BG8" s="83" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="BH8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BI8" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BJ8" s="110"/>
       <c r="BK8" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BL8" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BM8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BN8" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BO8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BP8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BQ8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BR8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BS8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BT8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BU8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BV8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BW8" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BX8" s="83" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="BY8" s="83"/>
       <c r="BZ8" s="83"/>
@@ -11648,244 +11739,244 @@
     </row>
     <row r="9" spans="1:97" ht="15.75">
       <c r="A9" s="80" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="B9" s="81" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="C9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="D9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="E9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="F9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="G9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="H9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="I9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="J9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="K9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="L9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="M9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="N9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="O9" s="86" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="P9" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Q9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="R9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="S9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="T9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="U9" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="V9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="W9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="X9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Y9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Z9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AA9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AB9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AC9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AD9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AE9" s="110"/>
       <c r="AF9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AG9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AH9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AI9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AJ9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AK9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AL9" s="110"/>
       <c r="AM9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AN9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AO9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AP9" s="110"/>
       <c r="AQ9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AR9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AS9" s="110"/>
       <c r="AT9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AU9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AV9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AW9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AX9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AY9" s="110"/>
       <c r="AZ9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BA9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BB9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BC9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BD9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BE9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BF9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BG9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BH9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BI9" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BJ9" s="110"/>
       <c r="BK9" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BL9" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BM9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BN9" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BO9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BP9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BQ9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BR9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BS9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BT9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BU9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BV9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BW9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BX9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BY9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BZ9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CA9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CB9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CC9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CD9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CE9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CF9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CG9" s="83"/>
       <c r="CH9" s="83"/>
@@ -11900,249 +11991,249 @@
       <c r="CQ9" s="83"/>
       <c r="CR9" s="83"/>
       <c r="CS9" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
     </row>
     <row r="10" spans="1:97" ht="15.75">
       <c r="A10" s="80" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="B10" s="81" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="C10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="D10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="E10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="F10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="G10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="H10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="I10" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="J10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="K10" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="L10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="M10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="N10" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="O10" s="83" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="P10" s="84" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="Q10" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="R10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="S10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="T10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="U10" s="84" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="V10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="W10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="X10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Y10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Z10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AA10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AB10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AC10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AD10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AE10" s="110"/>
       <c r="AF10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AG10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AH10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AI10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AJ10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AK10" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AL10" s="110"/>
       <c r="AM10" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AN10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AO10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AP10" s="110"/>
       <c r="AQ10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AR10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AS10" s="110"/>
       <c r="AT10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AU10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AV10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AW10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AX10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AY10" s="110"/>
       <c r="AZ10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BA10" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BB10" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BC10" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BD10" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BE10" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BF10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BG10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BH10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BI10" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BJ10" s="110"/>
       <c r="BK10" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BL10" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BM10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BN10" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BO10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BP10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BQ10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BR10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BS10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BT10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BU10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BV10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BW10" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BX10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BY10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BZ10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CA10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CB10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CC10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CD10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CE10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CF10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CG10" s="83"/>
       <c r="CH10" s="83"/>
@@ -12157,249 +12248,249 @@
       <c r="CQ10" s="83"/>
       <c r="CR10" s="83"/>
       <c r="CS10" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
     </row>
     <row r="11" spans="1:97" ht="15.75">
       <c r="A11" s="80" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="B11" s="81" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="C11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="D11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="E11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="F11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="G11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="H11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="I11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="J11" s="83" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="K11" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="L11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="M11" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="N11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="O11" s="83" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="P11" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Q11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="R11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="S11" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="T11" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="U11" s="84" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="V11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="W11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="X11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Y11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Z11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AA11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AB11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AC11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AD11" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AE11" s="110"/>
       <c r="AF11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AG11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AH11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AI11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AJ11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AK11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AL11" s="110"/>
       <c r="AM11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AN11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AO11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AP11" s="110"/>
       <c r="AQ11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AR11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AS11" s="110"/>
       <c r="AT11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AU11" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AV11" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AW11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AX11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AY11" s="110"/>
       <c r="AZ11" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BA11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BB11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BC11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BD11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BE11" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BF11" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BG11" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BH11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BI11" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BJ11" s="110"/>
       <c r="BK11" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BL11" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BM11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BN11" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BO11" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BP11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BQ11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BR11" s="83" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="BS11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BT11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BU11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BV11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BW11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BX11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BY11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BZ11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CA11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CB11" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="CC11" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="CD11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CE11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CF11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CG11" s="83"/>
       <c r="CH11" s="83"/>
@@ -12414,249 +12505,249 @@
       <c r="CQ11" s="83"/>
       <c r="CR11" s="83"/>
       <c r="CS11" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
     </row>
     <row r="12" spans="1:97" ht="15.75">
       <c r="A12" s="80" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="B12" s="81" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="C12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="D12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="E12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="F12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="G12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="H12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="I12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="J12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="K12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="L12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="M12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="N12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="O12" s="83" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="P12" s="84" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="Q12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="R12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="S12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="T12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="U12" s="84" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="V12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="W12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="X12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="Y12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="Z12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AA12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AB12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AC12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AD12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AE12" s="110"/>
       <c r="AF12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AG12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AH12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AI12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AJ12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AK12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AL12" s="110"/>
       <c r="AM12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AN12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AO12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AP12" s="110"/>
       <c r="AQ12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AR12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AS12" s="110"/>
       <c r="AT12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AU12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AV12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AW12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AX12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AY12" s="110"/>
       <c r="AZ12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BA12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BB12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BC12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BD12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BE12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BF12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BG12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BH12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BI12" s="84" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BJ12" s="110"/>
       <c r="BK12" s="84" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BL12" s="84" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BM12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BN12" s="84" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BO12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BP12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BQ12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BR12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BS12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BT12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BU12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BV12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BW12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BX12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BY12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="BZ12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="CA12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="CB12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CC12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="CD12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="CE12" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CF12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="CG12" s="83"/>
       <c r="CH12" s="83"/>
@@ -12671,249 +12762,249 @@
       <c r="CQ12" s="83"/>
       <c r="CR12" s="83"/>
       <c r="CS12" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
     </row>
     <row r="13" spans="1:97" ht="15.75">
       <c r="A13" s="80" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B13" s="81" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="C13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="D13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="E13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="F13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="G13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="H13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="I13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="J13" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="K13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="L13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="M13" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="N13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="O13" s="83" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="P13" s="84" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="Q13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="R13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="S13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="T13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="U13" s="84" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="V13" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="W13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="X13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="Y13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="Z13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AA13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AB13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AC13" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AD13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AE13" s="111"/>
       <c r="AF13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AG13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AH13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AI13" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="AJ13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AK13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AL13" s="111"/>
       <c r="AM13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AN13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AO13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AP13" s="111"/>
       <c r="AQ13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AR13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AS13" s="111"/>
       <c r="AT13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AU13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AV13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AW13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AX13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AY13" s="111"/>
       <c r="AZ13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BA13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BB13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BC13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BD13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BE13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BF13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BG13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BH13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BI13" s="84" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BJ13" s="111"/>
       <c r="BK13" s="84" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BL13" s="84" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BM13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BN13" s="84" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BO13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BP13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BQ13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BR13" s="83" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="BS13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BT13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BU13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BV13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BW13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BX13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BY13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="BZ13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="CA13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="CB13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="CC13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="CD13" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CE13" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CF13" s="83" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="CG13" s="83"/>
       <c r="CH13" s="83"/>
@@ -12928,7 +13019,7 @@
       <c r="CQ13" s="83"/>
       <c r="CR13" s="83"/>
       <c r="CS13" s="83" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -13947,7 +14038,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="25.5">
       <c r="A1" s="87" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="B1" s="87" t="s">
         <v>2</v>
@@ -13974,13 +14065,13 @@
         <v>12</v>
       </c>
       <c r="J1" s="91" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="K1" s="92" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="L1" s="90" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="M1" s="93"/>
       <c r="N1" s="93"/>
@@ -13999,10 +14090,10 @@
     </row>
     <row r="2" spans="1:26" ht="38.25">
       <c r="A2" s="94" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="B2" s="95" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="C2" s="96"/>
       <c r="D2" s="96" t="s">
@@ -14029,7 +14120,7 @@
       </c>
       <c r="K2" s="99"/>
       <c r="L2" s="100" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="M2" s="93"/>
       <c r="N2" s="93"/>
@@ -14048,13 +14139,13 @@
     </row>
     <row r="3" spans="1:26" ht="51">
       <c r="A3" s="94" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="B3" s="112" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="C3" s="101" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="D3" s="96" t="s">
         <v>110</v>
@@ -14076,7 +14167,7 @@
       </c>
       <c r="K3" s="97"/>
       <c r="L3" s="100" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="M3" s="102"/>
       <c r="N3" s="93"/>
@@ -14095,11 +14186,11 @@
     </row>
     <row r="4" spans="1:26" ht="51">
       <c r="A4" s="94" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="B4" s="110"/>
       <c r="C4" s="103" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="D4" s="96" t="s">
         <v>110</v>
@@ -14121,7 +14212,7 @@
       </c>
       <c r="K4" s="104"/>
       <c r="L4" s="107" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="M4" s="102"/>
       <c r="N4" s="93"/>
@@ -14140,13 +14231,13 @@
     </row>
     <row r="5" spans="1:26" ht="51">
       <c r="A5" s="94" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="B5" s="90" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="C5" s="96" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="D5" s="96" t="s">
         <v>110</v>
@@ -14168,7 +14259,7 @@
       </c>
       <c r="K5" s="97"/>
       <c r="L5" s="100" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="M5" s="102"/>
       <c r="N5" s="93"/>

</xml_diff>